<commit_message>
Update description for AXI2AHB
Update description for AXI2AHB
</commit_message>
<xml_diff>
--- a/doc/001_OpenVLSI_Resource.xlsx
+++ b/doc/001_OpenVLSI_Resource.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git\VLSIT_SOC_Starter\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2586FFDB-FD4E-4E27-A962-1669B11CDB15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{534174FB-E931-4D4D-B9EF-3A4EE710CE57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{B6857A90-25D4-4A67-8903-7C0067D27823}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="94">
   <si>
     <t>No.</t>
   </si>
@@ -546,12 +546,237 @@
   <si>
     <t>https://github.com/nguyenhong-hoa/WatchdogTimer.git</t>
   </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Support </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>outstading</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> but </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">not out-of-order --&gt; Maybe
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Responses always follow the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>order of issue</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+or only support a </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>single AXI ID</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+or </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>serialize</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> down to AHB
+Because there is a separate FIFO for ID --&gt; it uses method "serialize down to AHB"/ </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Support</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> multiple AXI ID/ Responses always follow the order of issue
+AXI </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>does not</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> support </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">lock/exclusive </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">accces (do not exsit AWLOCK/ARLOCK and HLOCK is tied 0)
+*Need exclusive access cases: 
+     Multi-core CPU
+     Share-memory DMA coordination
+     Modern OS kernels
+Features:
+AXI3 (exists WID) - AHB-Lite (No retry no Slip / HRESP chỉ có OKAY/ERROR)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <u/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Note</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> WID exists; no write interleaving logic detected. Likely for mapping only.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Bit width: 32-bit address/ 64-bit data.
+2 clock domain (hclk, aclk/ exsist 2-flop synchronizer/ FIFOs use gray code)</t>
+    </r>
+  </si>
+  <si>
+    <t>- Interface
+- features
+'- function
+Tool generate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">per README
+"The bridge does not implementAXI ID" and "Support FIXED/ INCR/ WRAP" -- &gt; Most likely AXI4
+</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -601,6 +826,22 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <u/>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -638,7 +879,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -672,6 +913,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1327,7 +1571,7 @@
       <c r="K20" s="7"/>
       <c r="L20" s="7"/>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" ht="346.2" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>4</v>
       </c>
@@ -1339,9 +1583,11 @@
         <v>60</v>
       </c>
       <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="F21" s="4" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" ht="67.2" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
@@ -1349,9 +1595,11 @@
         <v>61</v>
       </c>
       <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="F22" s="12" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" ht="67.2" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -1359,7 +1607,9 @@
         <v>62</v>
       </c>
       <c r="E23" s="1"/>
-      <c r="F23" s="1"/>
+      <c r="F23" s="4" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A24" s="1">

</xml_diff>